<commit_message>
Set Sheplik DeathRate to 0.3 (allometric scaling: predators die slower)
Allometric scaling law: natural mortality M ∝ W^(-0.25). Larger predators
have greater energy reserves and physiological buffering against chronic
stress, dying at roughly half the rate of smaller prey (McCoy & Gillooly
2008, Peterson & Wroblewski 1984).

- T1 Hexapod (prey): DeathRate = 0.6 (unchanged)
- T2 Sheplik (predator): DeathRate = 0.3 (was 0.6)

Updated in all 4 code locations (3 PopulateDefaultData + 1 ResetValues)
and both Excel sheets. Added allometric scaling citations to species
section comments.
</commit_message>
<xml_diff>
--- a/species.xlsx
+++ b/species.xlsx
@@ -1638,7 +1638,7 @@
         <v>0.3</v>
       </c>
       <c r="I5" s="8" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="J5" s="8" t="n">
         <v>0</v>
@@ -1747,7 +1747,7 @@
         <v>0.3</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>0</v>
@@ -1856,7 +1856,7 @@
         <v>0.3</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>0</v>
@@ -9301,7 +9301,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH7"/>
+  <dimension ref="A1:AH11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="14.43" customWidth="1" style="57" min="1" max="6"/>
@@ -9851,7 +9851,7 @@
         <v>0.3</v>
       </c>
       <c r="I5" s="52" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="J5" s="52" t="n">
         <v>0</v>
@@ -9961,7 +9961,7 @@
         <v>0.3</v>
       </c>
       <c r="I6" s="52" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="J6" s="52" t="n">
         <v>0</v>
@@ -10071,7 +10071,7 @@
         <v>0.3</v>
       </c>
       <c r="I7" s="52" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="J7" s="52" t="n">
         <v>0</v>
@@ -10153,6 +10153,10 @@
       </c>
       <c r="AH7" s="51" t="n"/>
     </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
     <row r="21" ht="15.75" customHeight="1" s="57"/>
     <row r="22" ht="15.75" customHeight="1" s="57"/>
     <row r="23" ht="15.75" customHeight="1" s="57"/>

</xml_diff>